<commit_message>
Auto: Add chapter "木瓜樹" (book: 三上)
</commit_message>
<xml_diff>
--- a/content-pipeline/inputs/book04/b04_ch14_final.xlsx
+++ b/content-pipeline/inputs/book04/b04_ch14_final.xlsx
@@ -553,7 +553,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>vines</t>
+          <t>vine</t>
         </is>
       </c>
     </row>
@@ -589,7 +589,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>serrated edges</t>
+          <t>serrated</t>
         </is>
       </c>
     </row>
@@ -625,7 +625,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>palm leaf fan</t>
+          <t>palm-leaf fan</t>
         </is>
       </c>
     </row>
@@ -649,7 +649,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>give off</t>
+          <t>emit</t>
         </is>
       </c>
     </row>
@@ -661,7 +661,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>light fragrance</t>
+          <t>faint fragrance</t>
         </is>
       </c>
     </row>
@@ -673,7 +673,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>pressed together</t>
+          <t>huddled together</t>
         </is>
       </c>
     </row>
@@ -697,7 +697,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>oblong</t>
+          <t>oval</t>
         </is>
       </c>
     </row>
@@ -865,7 +865,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>strong fragrance</t>
+          <t>rich aroma</t>
         </is>
       </c>
     </row>
@@ -877,7 +877,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>hot summer</t>
+          <t>scorching summer</t>
         </is>
       </c>
     </row>
@@ -957,7 +957,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>vines</t>
+          <t>vine</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -967,7 +967,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>在看到木瓜樹之前，我以為木瓜也是像西瓜一樣生長在地裏的，或者像黃瓜一樣長在藤蔓上。</t>
+          <t>在我以為木瓜像黃瓜一樣長在藤蔓上。</t>
         </is>
       </c>
     </row>
@@ -1023,7 +1023,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>serrated edges</t>
+          <t>serrated</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -1033,7 +1033,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>葉子帶有鋸齒，葉紋清晰可見。</t>
+          <t>葉子帶有鋸齒。</t>
         </is>
       </c>
     </row>
@@ -1055,7 +1055,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>葉子帶有鋸齒，葉紋清晰可見。</t>
+          <t>葉紋清晰可見。</t>
         </is>
       </c>
     </row>
@@ -1077,7 +1077,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>葉紋清晰可見。</t>
+          <t>葉子上的葉紋清晰可見。</t>
         </is>
       </c>
     </row>
@@ -1089,7 +1089,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>palm leaf fan</t>
+          <t>palm-leaf fan</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -1099,7 +1099,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>葉子好像一把把大蒲扇。</t>
+          <t>葉子像一把把大蒲扇。</t>
         </is>
       </c>
     </row>
@@ -1133,7 +1133,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>give off</t>
+          <t>emit</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -1155,7 +1155,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>light fragrance</t>
+          <t>faint fragrance</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -1165,7 +1165,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>木瓜樹的花散發着淡淡的清香。</t>
+          <t>花散發着淡淡的清香。</t>
         </is>
       </c>
     </row>
@@ -1177,7 +1177,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>pressed together</t>
+          <t>huddled together</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -1187,7 +1187,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>大大小小的木瓜緊緊地挨在一起。</t>
+          <t>木瓜緊緊地挨在一起。</t>
         </is>
       </c>
     </row>
@@ -1221,7 +1221,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>oblong</t>
+          <t>oval</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -1231,7 +1231,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>木瓜是長圓形的，好像一個個欖球。</t>
+          <t>木瓜是長圓形的。</t>
         </is>
       </c>
     </row>
@@ -1253,7 +1253,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>木瓜是長圓形的，好像一個個欖球。</t>
+          <t>木瓜好像一個個欖球。</t>
         </is>
       </c>
     </row>
@@ -1275,7 +1275,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>木瓜籽的外面有層透明的薄膜。</t>
+          <t>木瓜籽外面有層透明的薄膜。</t>
         </is>
       </c>
     </row>
@@ -1297,7 +1297,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>木瓜籽的外面有層透明的薄膜。</t>
+          <t>木瓜籽外面有層透明的薄膜。</t>
         </is>
       </c>
     </row>
@@ -1319,7 +1319,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>一粒粒好像烏黑發亮的小眼睛。</t>
+          <t>木瓜籽一粒粒好像烏黑發亮的小眼睛。</t>
         </is>
       </c>
     </row>
@@ -1385,7 +1385,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>木瓜素有『萬壽果』的稱號。</t>
+          <t>木瓜有『萬壽果』的稱號。</t>
         </is>
       </c>
     </row>
@@ -1407,7 +1407,7 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>木瓜含豐富維他命C。</t>
+          <t>木瓜含豐富的維他命C。</t>
         </is>
       </c>
     </row>
@@ -1429,7 +1429,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>木瓜含豐富維他命C、胡蘿蔔素以及蛋白酶。</t>
+          <t>木瓜含豐富的胡蘿蔔素。</t>
         </is>
       </c>
     </row>
@@ -1451,7 +1451,7 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>木瓜含豐富維他命C、胡蘿蔔素以及蛋白酶。</t>
+          <t>木瓜含豐富的蛋白酶。</t>
         </is>
       </c>
     </row>
@@ -1529,7 +1529,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>strong fragrance</t>
+          <t>rich aroma</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -1551,7 +1551,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>hot summer</t>
+          <t>scorching summer</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -1561,7 +1561,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>也是炎炎夏日中不錯的享受。</t>
+          <t>這也是炎炎夏日中不錯的享受。</t>
         </is>
       </c>
     </row>
@@ -1583,7 +1583,7 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>也是炎炎夏日中不錯的享受。</t>
+          <t>它是炎炎夏日中的享受。</t>
         </is>
       </c>
     </row>

</xml_diff>